<commit_message>
feat(schema): add polymorphic union types
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Quest.xlsx
+++ b/examples/showcase/data/Quest.xlsx
@@ -12,13 +12,14 @@
     <sheet name="MailTemplate" sheetId="3" r:id="rId3"/>
     <sheet name="MailReward" sheetId="4" r:id="rId4"/>
     <sheet name="Dialogue" sheetId="5" r:id="rId5"/>
+    <sheet name="EventRule" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="423">
   <si>
     <t>@table</t>
   </si>
@@ -1026,6 +1027,267 @@
   </si>
   <si>
     <t>["dialogue line 20-1","dialogue line 20-2"]</t>
+  </si>
+  <si>
+    <t>EventRule</t>
+  </si>
+  <si>
+    <t>ea4b96567144132b</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>condition</t>
+  </si>
+  <si>
+    <t>actions</t>
+  </si>
+  <si>
+    <t>union&lt;EventCondition&gt;</t>
+  </si>
+  <si>
+    <t>list&lt;union&lt;RewardAction&gt;&gt;</t>
+  </si>
+  <si>
+    <t>17001</t>
+  </si>
+  <si>
+    <t>Event Rule 1</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5002}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1007,"count":3 },{"type":"AddBuff","buff_id":6002,"duration":6 },{"type":"UnlockStage","stage_id":9002 }]</t>
+  </si>
+  <si>
+    <t>17002</t>
+  </si>
+  <si>
+    <t>Event Rule 2</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1005,"count":3}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1008,"count":4 },{"type":"AddBuff","buff_id":6003,"duration":7 },{"type":"UnlockStage","stage_id":9003 }]</t>
+  </si>
+  <si>
+    <t>17003</t>
+  </si>
+  <si>
+    <t>Event Rule 3</t>
+  </si>
+  <si>
+    <t>{"type":"LevelAtLeast","level":4}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1009,"count":5 },{"type":"AddBuff","buff_id":6004,"duration":8 },{"type":"UnlockStage","stage_id":9004 }]</t>
+  </si>
+  <si>
+    <t>17004</t>
+  </si>
+  <si>
+    <t>Event Rule 4</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5005}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1010,"count":2 },{"type":"AddBuff","buff_id":6005,"duration":9 },{"type":"UnlockStage","stage_id":9005 }]</t>
+  </si>
+  <si>
+    <t>17005</t>
+  </si>
+  <si>
+    <t>Event Rule 5</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1008,"count":1}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1011,"count":3 },{"type":"AddBuff","buff_id":6006,"duration":5 },{"type":"UnlockStage","stage_id":9006 }]</t>
+  </si>
+  <si>
+    <t>17006</t>
+  </si>
+  <si>
+    <t>Event Rule 6</t>
+  </si>
+  <si>
+    <t>{"type":"LevelAtLeast","level":7}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1012,"count":4 },{"type":"AddBuff","buff_id":6007,"duration":6 },{"type":"UnlockStage","stage_id":9007 }]</t>
+  </si>
+  <si>
+    <t>17007</t>
+  </si>
+  <si>
+    <t>Event Rule 7</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5008}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1013,"count":5 },{"type":"AddBuff","buff_id":6008,"duration":7 },{"type":"UnlockStage","stage_id":9008 }]</t>
+  </si>
+  <si>
+    <t>17008</t>
+  </si>
+  <si>
+    <t>Event Rule 8</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1011,"count":4}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1014,"count":2 },{"type":"AddBuff","buff_id":6009,"duration":8 },{"type":"UnlockStage","stage_id":9009 }]</t>
+  </si>
+  <si>
+    <t>17009</t>
+  </si>
+  <si>
+    <t>Event Rule 9</t>
+  </si>
+  <si>
+    <t>{"type":"LevelAtLeast","level":10}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1015,"count":3 },{"type":"AddBuff","buff_id":6010,"duration":9 },{"type":"UnlockStage","stage_id":9010 }]</t>
+  </si>
+  <si>
+    <t>17010</t>
+  </si>
+  <si>
+    <t>Event Rule 10</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5011}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1016,"count":4 },{"type":"AddBuff","buff_id":6011,"duration":5 },{"type":"UnlockStage","stage_id":9011 }]</t>
+  </si>
+  <si>
+    <t>17011</t>
+  </si>
+  <si>
+    <t>Event Rule 11</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1014,"count":2}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1017,"count":5 },{"type":"AddBuff","buff_id":6012,"duration":6 },{"type":"UnlockStage","stage_id":9012 }]</t>
+  </si>
+  <si>
+    <t>17012</t>
+  </si>
+  <si>
+    <t>Event Rule 12</t>
+  </si>
+  <si>
+    <t>{"type":"LevelAtLeast","level":13}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1018,"count":2 },{"type":"AddBuff","buff_id":6013,"duration":7 },{"type":"UnlockStage","stage_id":9013 }]</t>
+  </si>
+  <si>
+    <t>17013</t>
+  </si>
+  <si>
+    <t>Event Rule 13</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5014}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1019,"count":3 },{"type":"AddBuff","buff_id":6014,"duration":8 },{"type":"UnlockStage","stage_id":9014 }]</t>
+  </si>
+  <si>
+    <t>17014</t>
+  </si>
+  <si>
+    <t>Event Rule 14</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1017,"count":5}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1020,"count":4 },{"type":"AddBuff","buff_id":6015,"duration":9 },{"type":"UnlockStage","stage_id":9015 }]</t>
+  </si>
+  <si>
+    <t>17015</t>
+  </si>
+  <si>
+    <t>Event Rule 15</t>
+  </si>
+  <si>
+    <t>{"type":"LevelAtLeast","level":16}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1021,"count":5 },{"type":"AddBuff","buff_id":6016,"duration":5 },{"type":"UnlockStage","stage_id":9016 }]</t>
+  </si>
+  <si>
+    <t>17016</t>
+  </si>
+  <si>
+    <t>Event Rule 16</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5017}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1022,"count":2 },{"type":"AddBuff","buff_id":6017,"duration":6 },{"type":"UnlockStage","stage_id":9017 }]</t>
+  </si>
+  <si>
+    <t>17017</t>
+  </si>
+  <si>
+    <t>Event Rule 17</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1020,"count":3}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1023,"count":3 },{"type":"AddBuff","buff_id":6018,"duration":7 },{"type":"UnlockStage","stage_id":9018 }]</t>
+  </si>
+  <si>
+    <t>17018</t>
+  </si>
+  <si>
+    <t>Event Rule 18</t>
+  </si>
+  <si>
+    <t>{"type":"LevelAtLeast","level":19}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1024,"count":4 },{"type":"AddBuff","buff_id":6019,"duration":8 },{"type":"UnlockStage","stage_id":9019 }]</t>
+  </si>
+  <si>
+    <t>17019</t>
+  </si>
+  <si>
+    <t>Event Rule 19</t>
+  </si>
+  <si>
+    <t>{"type":"QuestCompleted","quest_id":5020}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1025,"count":5 },{"type":"AddBuff","buff_id":6020,"duration":9 },{"type":"UnlockStage","stage_id":9020 }]</t>
+  </si>
+  <si>
+    <t>17020</t>
+  </si>
+  <si>
+    <t>Event Rule 20</t>
+  </si>
+  <si>
+    <t>{"type":"HasItem","item_id":1023,"count":1}</t>
+  </si>
+  <si>
+    <t>[{"type":"AddItem","item_id":1026,"count":2 },{"type":"AddBuff","buff_id":6001,"duration":5 },{"type":"UnlockStage","stage_id":9021 }]</t>
   </si>
 </sst>
 </file>
@@ -4207,4 +4469,399 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D6" t="s">
+        <v>339</v>
+      </c>
+      <c r="E6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D7" t="s">
+        <v>339</v>
+      </c>
+      <c r="E7" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>341</v>
+      </c>
+      <c r="E8" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>343</v>
+      </c>
+      <c r="B11" t="s">
+        <v>344</v>
+      </c>
+      <c r="C11" t="s">
+        <v>345</v>
+      </c>
+      <c r="D11" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>347</v>
+      </c>
+      <c r="B12" t="s">
+        <v>348</v>
+      </c>
+      <c r="C12" t="s">
+        <v>349</v>
+      </c>
+      <c r="D12" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>351</v>
+      </c>
+      <c r="B13" t="s">
+        <v>352</v>
+      </c>
+      <c r="C13" t="s">
+        <v>353</v>
+      </c>
+      <c r="D13" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>355</v>
+      </c>
+      <c r="B14" t="s">
+        <v>356</v>
+      </c>
+      <c r="C14" t="s">
+        <v>357</v>
+      </c>
+      <c r="D14" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>359</v>
+      </c>
+      <c r="B15" t="s">
+        <v>360</v>
+      </c>
+      <c r="C15" t="s">
+        <v>361</v>
+      </c>
+      <c r="D15" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>363</v>
+      </c>
+      <c r="B16" t="s">
+        <v>364</v>
+      </c>
+      <c r="C16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D16" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>367</v>
+      </c>
+      <c r="B17" t="s">
+        <v>368</v>
+      </c>
+      <c r="C17" t="s">
+        <v>369</v>
+      </c>
+      <c r="D17" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B18" t="s">
+        <v>372</v>
+      </c>
+      <c r="C18" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>375</v>
+      </c>
+      <c r="B19" t="s">
+        <v>376</v>
+      </c>
+      <c r="C19" t="s">
+        <v>377</v>
+      </c>
+      <c r="D19" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>379</v>
+      </c>
+      <c r="B20" t="s">
+        <v>380</v>
+      </c>
+      <c r="C20" t="s">
+        <v>381</v>
+      </c>
+      <c r="D20" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>383</v>
+      </c>
+      <c r="B21" t="s">
+        <v>384</v>
+      </c>
+      <c r="C21" t="s">
+        <v>385</v>
+      </c>
+      <c r="D21" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>387</v>
+      </c>
+      <c r="B22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C22" t="s">
+        <v>389</v>
+      </c>
+      <c r="D22" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>391</v>
+      </c>
+      <c r="B23" t="s">
+        <v>392</v>
+      </c>
+      <c r="C23" t="s">
+        <v>393</v>
+      </c>
+      <c r="D23" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>395</v>
+      </c>
+      <c r="B24" t="s">
+        <v>396</v>
+      </c>
+      <c r="C24" t="s">
+        <v>397</v>
+      </c>
+      <c r="D24" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>399</v>
+      </c>
+      <c r="B25" t="s">
+        <v>400</v>
+      </c>
+      <c r="C25" t="s">
+        <v>401</v>
+      </c>
+      <c r="D25" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>403</v>
+      </c>
+      <c r="B26" t="s">
+        <v>404</v>
+      </c>
+      <c r="C26" t="s">
+        <v>405</v>
+      </c>
+      <c r="D26" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>407</v>
+      </c>
+      <c r="B27" t="s">
+        <v>408</v>
+      </c>
+      <c r="C27" t="s">
+        <v>409</v>
+      </c>
+      <c r="D27" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>411</v>
+      </c>
+      <c r="B28" t="s">
+        <v>412</v>
+      </c>
+      <c r="C28" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>415</v>
+      </c>
+      <c r="B29" t="s">
+        <v>416</v>
+      </c>
+      <c r="C29" t="s">
+        <v>417</v>
+      </c>
+      <c r="D29" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>419</v>
+      </c>
+      <c r="B30" t="s">
+        <v>420</v>
+      </c>
+      <c r="C30" t="s">
+        <v>421</v>
+      </c>
+      <c r="D30" t="s">
+        <v>422</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(showcase): generate excel data from templates
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Quest.xlsx
+++ b/examples/showcase/data/Quest.xlsx
@@ -18,6 +18,73 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+    <author>Sora</author>
+  </authors>
+  <commentList>
+    <comment ref="G7" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: start_pos
+Type: struct&lt;Vec3&gt;
+Scope: all
+Tuple fields: x: f32, y: f32, z: f32
+Required: yes</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H7" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Materialized from QuestReward child rows
+Field: rewards
+Type: list&lt;struct&lt;Reward&gt;&gt;
+Scope: all
+Aggregation: QuestReward.quest_id -&gt; id</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="426">
   <si>
@@ -1303,7 +1370,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1311,16 +1378,74 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F2937"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F3A4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9EEF5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D6E8F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE5EF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1328,12 +1453,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1630,687 +1788,735 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
+    <row r="6" spans="1:8" ht="6" customHeight="1"/>
+    <row r="7" spans="1:8" ht="24" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
+    <row r="12" spans="1:8" ht="42" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H12" t="s">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="5" t="s">
         <v>39</v>
       </c>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="5" t="s">
         <v>45</v>
       </c>
+      <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="G15" s="5"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="5" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
+      <c r="G16" s="5"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
+      <c r="G17" s="5"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
+      <c r="G18" s="5"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="5" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
+      <c r="G19" s="5"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="5" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
+      <c r="G20" s="5"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="5" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" t="s">
+      <c r="G21" s="5"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="5" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" t="s">
+      <c r="G22" s="5"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="5" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
+      <c r="G23" s="5"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="5" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" t="s">
+      <c r="G24" s="5"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="5" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" t="s">
+      <c r="G25" s="5"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="5" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" t="s">
+      <c r="G26" s="5"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="5" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" t="s">
+      <c r="G27" s="5"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="5" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" t="s">
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" t="s">
+      <c r="G29" s="5"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="5" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" t="s">
+      <c r="G30" s="5"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="5" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" t="s">
+      <c r="G31" s="5"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="5" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" t="s">
+      <c r="G32" s="5"/>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="5" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" t="s">
+      <c r="G33" s="5"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="5" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" t="s">
+      <c r="G34" s="5"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="5" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" t="s">
+      <c r="G35" s="5"/>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="5" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" t="s">
+      <c r="G36" s="5"/>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="5" t="s">
         <v>160</v>
       </c>
+      <c r="G37" s="5"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Main, Side, Daily" promptTitle="QuestType enum" prompt="Select a value from the dropdown." sqref="C13:C1012">
+      <formula1>"Main,Side,Daily"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2318,821 +2524,838 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E61"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="5" customWidth="1"/>
+    <col min="3" max="5" width="12.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B3" s="2"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
+    <row r="6" spans="1:5" ht="6" customHeight="1"/>
+    <row r="7" spans="1:5" ht="24" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" ht="42" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B14" t="s">
-        <v>173</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="B14" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="A17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B17" t="s">
-        <v>173</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B17" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="A18" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" t="s">
+      <c r="A19" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B19" t="s">
-        <v>173</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B19" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" t="s">
+      <c r="A20" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" t="s">
+      <c r="A21" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B21" t="s">
-        <v>173</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="B21" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="A22" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="A23" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B23" t="s">
-        <v>173</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="B23" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="A24" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="A25" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B25" t="s">
-        <v>173</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="B25" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" t="s">
+      <c r="A26" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" t="s">
+      <c r="A27" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B27" t="s">
-        <v>173</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="B27" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" t="s">
+      <c r="A28" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" t="s">
+      <c r="A29" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B29" t="s">
-        <v>173</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="B29" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" t="s">
+      <c r="A30" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" t="s">
+      <c r="A31" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B31" t="s">
-        <v>173</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="B31" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" t="s">
+      <c r="A32" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" t="s">
+      <c r="A33" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B33" t="s">
-        <v>173</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B33" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" t="s">
+      <c r="A34" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" t="s">
+      <c r="A35" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B35" t="s">
-        <v>173</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="B35" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" t="s">
+      <c r="A36" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" t="s">
+      <c r="A37" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B37" t="s">
-        <v>173</v>
-      </c>
-      <c r="C37" t="s">
+      <c r="B37" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" t="s">
+      <c r="A38" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" t="s">
+      <c r="A39" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B39" t="s">
-        <v>173</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="B39" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" t="s">
+      <c r="A40" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" t="s">
+      <c r="A41" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B41" t="s">
-        <v>173</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="B41" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" t="s">
+      <c r="A42" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" t="s">
+      <c r="A43" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B43" t="s">
-        <v>173</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B43" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C43" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" t="s">
+      <c r="A44" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" t="s">
+      <c r="A45" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B45" t="s">
-        <v>173</v>
-      </c>
-      <c r="C45" t="s">
+      <c r="B45" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" t="s">
+      <c r="A46" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:4">
-      <c r="A47" t="s">
+      <c r="A47" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B47" t="s">
-        <v>173</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="B47" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C47" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" t="s">
+      <c r="A48" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="49" spans="1:4">
-      <c r="A49" t="s">
+      <c r="A49" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B49" t="s">
-        <v>173</v>
-      </c>
-      <c r="C49" t="s">
+      <c r="B49" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" t="s">
+      <c r="A50" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" t="s">
+      <c r="A51" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B51" t="s">
-        <v>173</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="B51" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="52" spans="1:4">
-      <c r="A52" t="s">
+      <c r="A52" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="53" spans="1:4">
-      <c r="A53" t="s">
+      <c r="A53" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="B53" t="s">
-        <v>173</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="B53" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D53" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" t="s">
+      <c r="A54" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D54" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="55" spans="1:4">
-      <c r="A55" t="s">
+      <c r="A55" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B55" t="s">
-        <v>173</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="B55" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C55" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="56" spans="1:4">
-      <c r="A56" t="s">
+      <c r="A56" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="57" spans="1:4">
-      <c r="A57" t="s">
+      <c r="A57" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B57" t="s">
-        <v>173</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="B57" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C57" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" t="s">
+      <c r="A58" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" t="s">
+      <c r="A59" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B59" t="s">
-        <v>173</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="B59" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="60" spans="1:4">
-      <c r="A60" t="s">
+      <c r="A60" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:4">
-      <c r="A61" t="s">
+      <c r="A61" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B61" t="s">
-        <v>173</v>
-      </c>
-      <c r="C61" t="s">
+      <c r="B61" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C61" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D61" s="5" t="s">
         <v>176</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 9999." promptTitle="Integer range" prompt="Enter an integer from 1 to 9999." sqref="E13:E1012">
+      <formula1>1</formula1>
+      <formula2>9999</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3141,433 +3364,471 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="5" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
+    <row r="6" spans="1:6" ht="6" customHeight="1"/>
+    <row r="7" spans="1:6" ht="24" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
+    <row r="12" spans="1:6" ht="42" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>188</v>
       </c>
+      <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>192</v>
       </c>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>196</v>
       </c>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="E22" s="5"/>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="5" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="5" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="E24" s="5"/>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="5" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="5" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
+      <c r="E26" s="5"/>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="5" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" t="s">
+      <c r="E27" s="5"/>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="5" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" t="s">
+      <c r="E28" s="5"/>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="5" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" t="s">
+      <c r="E29" s="5"/>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="5" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" t="s">
+      <c r="E30" s="5"/>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="5" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" t="s">
+      <c r="E31" s="5"/>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="5" t="s">
         <v>247</v>
       </c>
+      <c r="E32" s="5"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: System, Event, Compensation" promptTitle="MailType enum" prompt="Select a value from the dropdown." sqref="C13:C1012">
+      <formula1>"System,Event,Compensation"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3576,691 +3837,702 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="5" customWidth="1"/>
+    <col min="3" max="5" width="12.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B3" s="2"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
+    <row r="6" spans="1:5" ht="6" customHeight="1"/>
+    <row r="7" spans="1:5" ht="24" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" ht="42" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B14" t="s">
-        <v>173</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="B14" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B16" t="s">
-        <v>173</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="B16" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="A17" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="A18" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B18" t="s">
-        <v>173</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B18" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" t="s">
+      <c r="A19" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" t="s">
+      <c r="A20" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B20" t="s">
-        <v>173</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="B20" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" t="s">
+      <c r="A21" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="A22" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="B22" t="s">
-        <v>173</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="B22" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="A23" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="A24" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B24" t="s">
-        <v>173</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="B24" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="A25" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" t="s">
+      <c r="A26" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B26" t="s">
-        <v>173</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="B26" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" t="s">
+      <c r="A27" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" t="s">
+      <c r="A28" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="B28" t="s">
-        <v>173</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="B28" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" t="s">
+      <c r="A29" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" t="s">
+      <c r="A30" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="B30" t="s">
-        <v>173</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="B30" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" t="s">
+      <c r="A31" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" t="s">
+      <c r="A32" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B32" t="s">
-        <v>173</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="B32" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" t="s">
+      <c r="A33" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" t="s">
+      <c r="A34" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B34" t="s">
-        <v>173</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="B34" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" t="s">
+      <c r="A35" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" t="s">
+      <c r="A36" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B36" t="s">
-        <v>173</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="B36" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" t="s">
+      <c r="A37" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" t="s">
+      <c r="A38" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B38" t="s">
-        <v>173</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="B38" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" t="s">
+      <c r="A39" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" t="s">
+      <c r="A40" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B40" t="s">
-        <v>173</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="B40" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" t="s">
+      <c r="A41" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" t="s">
+      <c r="A42" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="B42" t="s">
-        <v>173</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="B42" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" t="s">
+      <c r="A43" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" t="s">
+      <c r="A44" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="B44" t="s">
-        <v>173</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="B44" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" t="s">
+      <c r="A45" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" t="s">
+      <c r="A46" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B46" t="s">
-        <v>173</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="B46" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:4">
-      <c r="A47" t="s">
+      <c r="A47" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" t="s">
+      <c r="A48" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="B48" t="s">
-        <v>173</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="B48" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="49" spans="1:4">
-      <c r="A49" t="s">
+      <c r="A49" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" t="s">
+      <c r="A50" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="B50" t="s">
-        <v>173</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="B50" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" t="s">
+      <c r="A51" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="52" spans="1:4">
-      <c r="A52" t="s">
+      <c r="A52" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="B52" t="s">
-        <v>173</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="B52" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" s="5" t="s">
         <v>176</v>
       </c>
     </row>
@@ -4273,339 +4545,347 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="12.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="6" spans="1:4" ht="6" customHeight="1"/>
+    <row r="7" spans="1:4" ht="24" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
+    <row r="12" spans="1:4" ht="42" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" t="s">
+      <c r="A17" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" t="s">
+      <c r="A18" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" t="s">
+      <c r="A19" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" t="s">
+      <c r="A20" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" t="s">
+      <c r="A21" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" t="s">
+      <c r="A22" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" t="s">
+      <c r="A23" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" t="s">
+      <c r="A24" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="25" spans="1:3">
-      <c r="A25" t="s">
+      <c r="A25" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="26" spans="1:3">
-      <c r="A26" t="s">
+      <c r="A26" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" t="s">
+      <c r="A27" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>321</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="28" spans="1:3">
-      <c r="A28" t="s">
+      <c r="A28" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="29" spans="1:3">
-      <c r="A29" t="s">
+      <c r="A29" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="5" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="30" spans="1:3">
-      <c r="A30" t="s">
+      <c r="A30" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="5" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="31" spans="1:3">
-      <c r="A31" t="s">
+      <c r="A31" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="5" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" t="s">
+      <c r="A32" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="5" t="s">
         <v>337</v>
       </c>
     </row>
@@ -4618,414 +4898,425 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
+    <row r="6" spans="1:5" ht="6" customHeight="1"/>
+    <row r="7" spans="1:5" ht="24" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" ht="42" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="A17" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="A18" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" t="s">
+      <c r="A19" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" t="s">
+      <c r="A20" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" t="s">
+      <c r="A21" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="A22" s="5" t="s">
         <v>382</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="A23" s="5" t="s">
         <v>386</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="5" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="A24" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="5" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="A25" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>396</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="5" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" t="s">
+      <c r="A26" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>399</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="5" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" t="s">
+      <c r="A27" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="5" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" t="s">
+      <c r="A28" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>407</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="5" t="s">
         <v>409</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" t="s">
+      <c r="A29" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="5" t="s">
         <v>413</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" t="s">
+      <c r="A30" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="5" t="s">
         <v>416</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="5" t="s">
         <v>417</v>
       </c>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" t="s">
+      <c r="A31" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="5" t="s">
         <v>420</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="5" t="s">
         <v>421</v>
       </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" t="s">
+      <c r="A32" s="5" t="s">
         <v>422</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="5" t="s">
         <v>424</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="5" t="s">
         <v>425</v>
       </c>
     </row>

</xml_diff>